<commit_message>
Record external JobKorea count
</commit_message>
<xml_diff>
--- a/data/job_post_counts.xlsx
+++ b/data/job_post_counts.xlsx
@@ -81,12 +81,12 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$141</c:f>
+              <c:f>Data!$A$2:$A$142</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$C$2:$C$141</c:f>
+              <c:f>Data!$C$2:$C$142</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -154,12 +154,12 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>WeeklyOHLC!$A$2:$A$21</c:f>
+              <c:f>WeeklyOHLC!$A$2:$A$22</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>WeeklyOHLC!$B$2:$B$21</c:f>
+              <c:f>WeeklyOHLC!$B$2:$B$22</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -171,12 +171,12 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>WeeklyOHLC!$A$2:$A$21</c:f>
+              <c:f>WeeklyOHLC!$A$2:$A$22</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>WeeklyOHLC!$C$2:$C$21</c:f>
+              <c:f>WeeklyOHLC!$C$2:$C$22</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -188,12 +188,12 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>WeeklyOHLC!$A$2:$A$21</c:f>
+              <c:f>WeeklyOHLC!$A$2:$A$22</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>WeeklyOHLC!$D$2:$D$21</c:f>
+              <c:f>WeeklyOHLC!$D$2:$D$22</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -205,12 +205,12 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>WeeklyOHLC!$A$2:$A$21</c:f>
+              <c:f>WeeklyOHLC!$A$2:$A$22</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>WeeklyOHLC!$E$2:$E$21</c:f>
+              <c:f>WeeklyOHLC!$E$2:$E$22</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -4568,8 +4568,38 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-14 09:00:36</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C142">
+        <v>193649</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>parsed joblist hdnGICnt</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>https://www.jobkorea.co.kr/recruit/joblist?menucode=local&amp;localorder=1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F141"/>
+  <autoFilter ref="A1:F142"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4996,8 +5026,27 @@
         <v>198797</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B22">
+        <v>193649</v>
+      </c>
+      <c r="C22">
+        <v>193649</v>
+      </c>
+      <c r="D22">
+        <v>193649</v>
+      </c>
+      <c r="E22">
+        <v>193649</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E21"/>
+  <autoFilter ref="A1:E22"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>